<commit_message>
Fix database concurrency, WAL corruption, and SII csv parser
</commit_message>
<xml_diff>
--- a/REGISTRO FACTURAS.xlsx
+++ b/REGISTRO FACTURAS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c786fff28ee952f5/Documentos/PROYECTOS/BD SENIOR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="705" documentId="8_{FABFBFA3-4FFC-4BCB-A04F-FE0D25E4DD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66D8171E-29BC-4FFE-ABE8-31B55D47E742}"/>
+  <xr:revisionPtr revIDLastSave="750" documentId="8_{FABFBFA3-4FFC-4BCB-A04F-FE0D25E4DD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86A931CC-6070-4CF9-A5BD-07D77C124CAF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9457EB46-FD10-4BB2-A776-79809D00B0E2}"/>
+    <workbookView minimized="1" xWindow="1668" yWindow="2916" windowWidth="15468" windowHeight="9852" xr2:uid="{9457EB46-FD10-4BB2-A776-79809D00B0E2}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE 26" sheetId="3" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="143">
   <si>
     <t>Nro</t>
   </si>
@@ -491,6 +491,12 @@
   </si>
   <si>
     <t>F29 (IVA, IMPUESTO A LA RENTA ($85.371), RETENCIÓN BOLETA HONORARIOS ($539.823), PPM, ETC.</t>
+  </si>
+  <si>
+    <t>2026/08</t>
+  </si>
+  <si>
+    <t>2026/09</t>
   </si>
 </sst>
 </file>
@@ -1263,7 +1269,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1621,6 +1627,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1990,7 +2002,7 @@
     <col min="5" max="5" width="14.33203125" style="100" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.6640625" style="1" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" style="15" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" style="2" bestFit="1" customWidth="1"/>
@@ -2734,7 +2746,7 @@
         <v>938046787</v>
       </c>
       <c r="F12" s="72">
-        <f t="shared" ref="F12:F17" si="4">H12/1.19</f>
+        <f t="shared" ref="F12:F22" si="4">H12/1.19</f>
         <v>7035351.260504202</v>
       </c>
       <c r="G12" s="72">
@@ -3119,14 +3131,32 @@
       <c r="X17" s="17"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A18" s="22"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="99"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="24"/>
+      <c r="A18" s="33">
+        <v>46248</v>
+      </c>
+      <c r="B18" s="34">
+        <v>20</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" s="96">
+        <v>564482110</v>
+      </c>
+      <c r="F18" s="72">
+        <f t="shared" si="4"/>
+        <v>4233615.9663865548</v>
+      </c>
+      <c r="G18" s="72">
+        <f t="shared" ref="G18:G22" si="7">H18-F18</f>
+        <v>804387.03361344524</v>
+      </c>
+      <c r="H18" s="40">
+        <v>5038003</v>
+      </c>
       <c r="J18" s="51">
         <v>46106</v>
       </c>
@@ -3143,11 +3173,11 @@
         <v>66</v>
       </c>
       <c r="O18" s="10">
-        <f t="shared" ref="O18" si="7">Q18/1.19</f>
+        <f t="shared" ref="O18" si="8">Q18/1.19</f>
         <v>747882.3529411765</v>
       </c>
       <c r="P18" s="10">
-        <f t="shared" ref="P18" si="8">Q18-O18</f>
+        <f t="shared" ref="P18" si="9">Q18-O18</f>
         <v>142097.6470588235</v>
       </c>
       <c r="Q18" s="52">
@@ -3167,14 +3197,32 @@
       </c>
     </row>
     <row r="19" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="22"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="99"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="24"/>
+      <c r="A19" s="22">
+        <v>46248</v>
+      </c>
+      <c r="B19" s="5">
+        <v>21</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E19" s="97">
+        <v>2531508878.0535293</v>
+      </c>
+      <c r="F19" s="44">
+        <f t="shared" si="4"/>
+        <v>1233316.8067226892</v>
+      </c>
+      <c r="G19" s="44">
+        <f t="shared" si="7"/>
+        <v>234330.19327731081</v>
+      </c>
+      <c r="H19" s="24">
+        <v>1467647</v>
+      </c>
       <c r="J19" s="75">
         <v>46106</v>
       </c>
@@ -3211,15 +3259,33 @@
       </c>
       <c r="X19" s="17"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A20" s="22"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="99"/>
-      <c r="F20" s="43"/>
-      <c r="G20" s="43"/>
-      <c r="H20" s="24"/>
+    <row r="20" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="36">
+        <v>46248</v>
+      </c>
+      <c r="B20" s="37">
+        <v>22</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>141</v>
+      </c>
+      <c r="E20" s="98">
+        <v>7114939744.1653738</v>
+      </c>
+      <c r="F20" s="73">
+        <f t="shared" si="4"/>
+        <v>3669625.2100840337</v>
+      </c>
+      <c r="G20" s="73">
+        <f t="shared" si="7"/>
+        <v>697228.78991596634</v>
+      </c>
+      <c r="H20" s="39">
+        <v>4366854</v>
+      </c>
       <c r="J20" s="33">
         <v>46137</v>
       </c>
@@ -3253,14 +3319,32 @@
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A21" s="22"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="99"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="24"/>
+      <c r="A21" s="33">
+        <v>46279</v>
+      </c>
+      <c r="B21" s="34">
+        <v>23</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="E21" s="96">
+        <v>2608888377.6156387</v>
+      </c>
+      <c r="F21" s="72">
+        <f t="shared" si="4"/>
+        <v>1283135.2941176472</v>
+      </c>
+      <c r="G21" s="72">
+        <f t="shared" si="7"/>
+        <v>243795.70588235278</v>
+      </c>
+      <c r="H21" s="40">
+        <v>1526931</v>
+      </c>
       <c r="J21" s="22">
         <v>46122</v>
       </c>
@@ -3284,15 +3368,33 @@
       <c r="U21" s="6"/>
       <c r="V21" s="24"/>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A22" s="22"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="99"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="24"/>
+    <row r="22" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="36">
+        <v>46279</v>
+      </c>
+      <c r="B22" s="37">
+        <v>24</v>
+      </c>
+      <c r="C22" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22" s="98">
+        <v>7259546032.558651</v>
+      </c>
+      <c r="F22" s="73">
+        <f t="shared" si="4"/>
+        <v>3634136.9747899161</v>
+      </c>
+      <c r="G22" s="73">
+        <f t="shared" si="7"/>
+        <v>690486.02521008393</v>
+      </c>
+      <c r="H22" s="39">
+        <v>4324623</v>
+      </c>
       <c r="J22" s="22">
         <v>46122</v>
       </c>
@@ -3319,14 +3421,14 @@
       <c r="X22" s="17"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A23" s="22"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="99"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="24"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="120"/>
+      <c r="F23" s="121"/>
+      <c r="G23" s="121"/>
+      <c r="H23" s="71"/>
       <c r="J23" s="22">
         <v>46141</v>
       </c>
@@ -3443,11 +3545,11 @@
         <v>66</v>
       </c>
       <c r="O26" s="10">
-        <f t="shared" ref="O26:O27" si="9">Q26/1.19</f>
+        <f t="shared" ref="O26:O27" si="10">Q26/1.19</f>
         <v>80470.588235294126</v>
       </c>
       <c r="P26" s="10">
-        <f t="shared" ref="P26:P28" si="10">Q26-O26</f>
+        <f t="shared" ref="P26:P28" si="11">Q26-O26</f>
         <v>15289.411764705874</v>
       </c>
       <c r="Q26" s="23">
@@ -3483,11 +3585,11 @@
         <v>66</v>
       </c>
       <c r="O27" s="10">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>47210.08403361345</v>
       </c>
       <c r="P27" s="10">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>8969.9159663865503</v>
       </c>
       <c r="Q27" s="23">
@@ -3521,11 +3623,11 @@
         <v>65</v>
       </c>
       <c r="O28" s="10">
-        <f t="shared" ref="O28" si="11">Q28/1.19</f>
+        <f t="shared" ref="O28" si="12">Q28/1.19</f>
         <v>155701.68067226891</v>
       </c>
       <c r="P28" s="10">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>29583.319327731093</v>
       </c>
       <c r="Q28" s="23">
@@ -3791,11 +3893,11 @@
         <v>111</v>
       </c>
       <c r="O36" s="10">
-        <f t="shared" ref="O36" si="12">Q36/1.19</f>
+        <f t="shared" ref="O36" si="13">Q36/1.19</f>
         <v>131050.42016806723</v>
       </c>
       <c r="P36" s="10">
-        <f t="shared" ref="P36" si="13">Q36-O36</f>
+        <f t="shared" ref="P36" si="14">Q36-O36</f>
         <v>24899.579831932773</v>
       </c>
       <c r="Q36" s="23">
@@ -3865,11 +3967,11 @@
         <v>65</v>
       </c>
       <c r="O38" s="64">
-        <f t="shared" ref="O38" si="14">Q38/1.19</f>
+        <f t="shared" ref="O38" si="15">Q38/1.19</f>
         <v>302278.99159663869</v>
       </c>
       <c r="P38" s="64">
-        <f t="shared" ref="P38" si="15">Q38-O38</f>
+        <f t="shared" ref="P38" si="16">Q38-O38</f>
         <v>57433.008403361309</v>
       </c>
       <c r="Q38" s="29">
@@ -3933,11 +4035,11 @@
         <v>111</v>
       </c>
       <c r="O40" s="10">
-        <f t="shared" ref="O40:O41" si="16">Q40/1.19</f>
+        <f t="shared" ref="O40:O41" si="17">Q40/1.19</f>
         <v>37470.588235294119</v>
       </c>
       <c r="P40" s="10">
-        <f t="shared" ref="P40:P41" si="17">Q40-O40</f>
+        <f t="shared" ref="P40:P41" si="18">Q40-O40</f>
         <v>7119.4117647058811</v>
       </c>
       <c r="Q40" s="23">
@@ -3969,11 +4071,11 @@
         <v>111</v>
       </c>
       <c r="O41" s="10">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>42546.218487394959</v>
       </c>
       <c r="P41" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>8083.7815126050409</v>
       </c>
       <c r="Q41" s="23">
@@ -4494,15 +4596,15 @@
       <c r="E61" s="67"/>
       <c r="F61" s="21">
         <f>SUM(F3:F24)</f>
-        <v>76158635.294117659</v>
+        <v>90212465.5462185</v>
       </c>
       <c r="G61" s="21">
         <f>SUM(G3:G24)</f>
-        <v>14470140.70588235</v>
+        <v>17140368.453781508</v>
       </c>
       <c r="H61" s="21">
         <f>SUM(H3:H24)</f>
-        <v>90628776</v>
+        <v>107352834</v>
       </c>
       <c r="J61" s="115"/>
       <c r="K61" s="116"/>

</xml_diff>

<commit_message>
Fix GCS cloud sync: add live status banner, drag-and-drop Excel sync, force hot upload, and error alerts
</commit_message>
<xml_diff>
--- a/REGISTRO FACTURAS.xlsx
+++ b/REGISTRO FACTURAS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c786fff28ee952f5/Documentos/PROYECTOS/BD SENIOR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="750" documentId="8_{FABFBFA3-4FFC-4BCB-A04F-FE0D25E4DD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86A931CC-6070-4CF9-A5BD-07D77C124CAF}"/>
+  <xr:revisionPtr revIDLastSave="790" documentId="8_{FABFBFA3-4FFC-4BCB-A04F-FE0D25E4DD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C559655-12EE-480B-ACE8-B953520805BE}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1668" yWindow="2916" windowWidth="15468" windowHeight="9852" xr2:uid="{9457EB46-FD10-4BB2-A776-79809D00B0E2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9457EB46-FD10-4BB2-A776-79809D00B0E2}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE 26" sheetId="3" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="145">
   <si>
     <t>Nro</t>
   </si>
@@ -497,14 +497,21 @@
   </si>
   <si>
     <t>2026/09</t>
+  </si>
+  <si>
+    <t>2026/10</t>
+  </si>
+  <si>
+    <t>PIS_836</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="42" formatCode="_ &quot;$&quot;* #,##0_ ;_ &quot;$&quot;* \-#,##0_ ;_ &quot;$&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -1265,11 +1272,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1580,6 +1588,24 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1628,14 +1654,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Millares [0]" xfId="2" builtinId="6"/>
     <cellStyle name="Moneda [0]" xfId="1" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1992,7 +2013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2822C60C-6EB5-4419-A8A5-7CA3B8AEE8EE}">
-  <dimension ref="A1:Y69"/>
+  <dimension ref="A1:Y70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1"/>
@@ -2000,7 +2021,7 @@
     <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.33203125" style="100" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="14.109375" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.6640625" style="1" customWidth="1"/>
@@ -2024,41 +2045,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="16" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="110" t="s">
+      <c r="A1" s="116" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="112" t="s">
+      <c r="B1" s="118" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="114"/>
-      <c r="J1" s="110" t="s">
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="120"/>
+      <c r="J1" s="116" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="104" t="s">
+      <c r="K1" s="110" t="s">
         <v>59</v>
       </c>
-      <c r="L1" s="105"/>
-      <c r="M1" s="105"/>
-      <c r="N1" s="105"/>
-      <c r="O1" s="105"/>
-      <c r="P1" s="105"/>
-      <c r="Q1" s="106"/>
-      <c r="S1" s="110" t="s">
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="112"/>
+      <c r="S1" s="116" t="s">
         <v>38</v>
       </c>
-      <c r="T1" s="104" t="s">
+      <c r="T1" s="110" t="s">
         <v>63</v>
       </c>
-      <c r="U1" s="105"/>
-      <c r="V1" s="106"/>
+      <c r="U1" s="111"/>
+      <c r="V1" s="112"/>
     </row>
     <row r="2" spans="1:25" s="16" customFormat="1" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="111"/>
+      <c r="A2" s="117"/>
       <c r="B2" s="18" t="s">
         <v>39</v>
       </c>
@@ -2080,7 +2101,7 @@
       <c r="H2" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="111"/>
+      <c r="J2" s="117"/>
       <c r="K2" s="18" t="s">
         <v>39</v>
       </c>
@@ -2102,7 +2123,7 @@
       <c r="Q2" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="S2" s="117"/>
+      <c r="S2" s="123"/>
       <c r="T2" s="30" t="s">
         <v>40</v>
       </c>
@@ -3421,14 +3442,32 @@
       <c r="X22" s="17"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A23" s="27"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="120"/>
-      <c r="F23" s="121"/>
-      <c r="G23" s="121"/>
-      <c r="H23" s="71"/>
+      <c r="A23" s="33">
+        <v>46309</v>
+      </c>
+      <c r="B23" s="34">
+        <v>29</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="E23" s="106">
+        <v>1335309005</v>
+      </c>
+      <c r="F23" s="72">
+        <f t="shared" ref="F23:F26" si="10">H23/1.19</f>
+        <v>10014817.647058824</v>
+      </c>
+      <c r="G23" s="72">
+        <f t="shared" ref="G23:G26" si="11">H23-F23</f>
+        <v>1902815.3529411759</v>
+      </c>
+      <c r="H23" s="40">
+        <v>11917633</v>
+      </c>
       <c r="J23" s="22">
         <v>46141</v>
       </c>
@@ -3453,14 +3492,32 @@
       <c r="V23" s="24"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" s="22"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="99"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="24"/>
+      <c r="A24" s="27">
+        <v>46309</v>
+      </c>
+      <c r="B24" s="46">
+        <v>26</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E24" s="104">
+        <v>284251105.63401383</v>
+      </c>
+      <c r="F24" s="44">
+        <f t="shared" ref="F24" si="12">H24/1.19</f>
+        <v>260924.36974789918</v>
+      </c>
+      <c r="G24" s="44">
+        <f t="shared" ref="G24" si="13">H24-F24</f>
+        <v>49575.630252100818</v>
+      </c>
+      <c r="H24" s="71">
+        <v>310500</v>
+      </c>
       <c r="J24" s="22">
         <v>46141</v>
       </c>
@@ -3485,14 +3542,32 @@
       <c r="V24" s="24"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A25" s="22"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="99"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="24"/>
+      <c r="A25" s="27">
+        <v>46309</v>
+      </c>
+      <c r="B25" s="5">
+        <v>27</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25" s="99">
+        <v>2679907837.7460337</v>
+      </c>
+      <c r="F25" s="44">
+        <f t="shared" si="10"/>
+        <v>1276989.0756302522</v>
+      </c>
+      <c r="G25" s="44">
+        <f t="shared" si="11"/>
+        <v>242627.92436974775</v>
+      </c>
+      <c r="H25" s="24">
+        <v>1519617</v>
+      </c>
       <c r="J25" s="22">
         <v>46141</v>
       </c>
@@ -3520,15 +3595,33 @@
       <c r="U25" s="6"/>
       <c r="V25" s="24"/>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A26" s="22"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="99"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="24"/>
+    <row r="26" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="109">
+        <v>46309</v>
+      </c>
+      <c r="B26" s="37">
+        <v>28</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26" s="107">
+        <v>7503144813.8048859</v>
+      </c>
+      <c r="F26" s="73">
+        <f t="shared" si="10"/>
+        <v>3332650.4201680673</v>
+      </c>
+      <c r="G26" s="73">
+        <f t="shared" si="11"/>
+        <v>633203.57983193267</v>
+      </c>
+      <c r="H26" s="39">
+        <v>3965854</v>
+      </c>
       <c r="J26" s="22">
         <v>46138</v>
       </c>
@@ -3545,11 +3638,11 @@
         <v>66</v>
       </c>
       <c r="O26" s="10">
-        <f t="shared" ref="O26:O27" si="10">Q26/1.19</f>
+        <f t="shared" ref="O26:O27" si="14">Q26/1.19</f>
         <v>80470.588235294126</v>
       </c>
       <c r="P26" s="10">
-        <f t="shared" ref="P26:P28" si="11">Q26-O26</f>
+        <f t="shared" ref="P26:P28" si="15">Q26-O26</f>
         <v>15289.411764705874</v>
       </c>
       <c r="Q26" s="23">
@@ -3561,14 +3654,14 @@
       <c r="V26" s="24"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A27" s="22"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="99"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="24"/>
+      <c r="A27" s="27"/>
+      <c r="B27" s="46"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="104"/>
+      <c r="F27" s="105"/>
+      <c r="G27" s="105"/>
+      <c r="H27" s="71"/>
       <c r="J27" s="22">
         <v>46138</v>
       </c>
@@ -3585,11 +3678,11 @@
         <v>66</v>
       </c>
       <c r="O27" s="10">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>47210.08403361345</v>
       </c>
       <c r="P27" s="10">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>8969.9159663865503</v>
       </c>
       <c r="Q27" s="23">
@@ -3623,11 +3716,11 @@
         <v>65</v>
       </c>
       <c r="O28" s="10">
-        <f t="shared" ref="O28" si="12">Q28/1.19</f>
+        <f t="shared" ref="O28" si="16">Q28/1.19</f>
         <v>155701.68067226891</v>
       </c>
       <c r="P28" s="10">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>29583.319327731093</v>
       </c>
       <c r="Q28" s="23">
@@ -3893,11 +3986,11 @@
         <v>111</v>
       </c>
       <c r="O36" s="10">
-        <f t="shared" ref="O36" si="13">Q36/1.19</f>
+        <f t="shared" ref="O36" si="17">Q36/1.19</f>
         <v>131050.42016806723</v>
       </c>
       <c r="P36" s="10">
-        <f t="shared" ref="P36" si="14">Q36-O36</f>
+        <f t="shared" ref="P36" si="18">Q36-O36</f>
         <v>24899.579831932773</v>
       </c>
       <c r="Q36" s="23">
@@ -3967,11 +4060,11 @@
         <v>65</v>
       </c>
       <c r="O38" s="64">
-        <f t="shared" ref="O38" si="15">Q38/1.19</f>
+        <f t="shared" ref="O38" si="19">Q38/1.19</f>
         <v>302278.99159663869</v>
       </c>
       <c r="P38" s="64">
-        <f t="shared" ref="P38" si="16">Q38-O38</f>
+        <f t="shared" ref="P38" si="20">Q38-O38</f>
         <v>57433.008403361309</v>
       </c>
       <c r="Q38" s="29">
@@ -4035,11 +4128,11 @@
         <v>111</v>
       </c>
       <c r="O40" s="10">
-        <f t="shared" ref="O40:O41" si="17">Q40/1.19</f>
+        <f t="shared" ref="O40:O41" si="21">Q40/1.19</f>
         <v>37470.588235294119</v>
       </c>
       <c r="P40" s="10">
-        <f t="shared" ref="P40:P41" si="18">Q40-O40</f>
+        <f t="shared" ref="P40:P41" si="22">Q40-O40</f>
         <v>7119.4117647058811</v>
       </c>
       <c r="Q40" s="23">
@@ -4071,11 +4164,11 @@
         <v>111</v>
       </c>
       <c r="O41" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="21"/>
         <v>42546.218487394959</v>
       </c>
       <c r="P41" s="10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="22"/>
         <v>8083.7815126050409</v>
       </c>
       <c r="Q41" s="23">
@@ -4589,27 +4682,18 @@
       <c r="V60" s="24"/>
     </row>
     <row r="61" spans="1:22" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="115"/>
-      <c r="B61" s="116"/>
-      <c r="C61" s="116"/>
-      <c r="D61" s="116"/>
-      <c r="E61" s="67"/>
-      <c r="F61" s="21">
-        <f>SUM(F3:F24)</f>
-        <v>90212465.5462185</v>
-      </c>
-      <c r="G61" s="21">
-        <f>SUM(G3:G24)</f>
-        <v>17140368.453781508</v>
-      </c>
-      <c r="H61" s="21">
-        <f>SUM(H3:H24)</f>
-        <v>107352834</v>
-      </c>
-      <c r="J61" s="115"/>
-      <c r="K61" s="116"/>
-      <c r="L61" s="116"/>
-      <c r="M61" s="116"/>
+      <c r="A61" s="22"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="99"/>
+      <c r="F61" s="43"/>
+      <c r="G61" s="43"/>
+      <c r="H61" s="24"/>
+      <c r="J61" s="121"/>
+      <c r="K61" s="122"/>
+      <c r="L61" s="122"/>
+      <c r="M61" s="122"/>
       <c r="N61" s="20"/>
       <c r="O61" s="67"/>
       <c r="P61" s="67"/>
@@ -4617,22 +4701,42 @@
         <f>SUM(Q3:Q60)</f>
         <v>37859227</v>
       </c>
-      <c r="S61" s="107"/>
-      <c r="T61" s="108"/>
-      <c r="U61" s="109"/>
+      <c r="S61" s="113"/>
+      <c r="T61" s="114"/>
+      <c r="U61" s="115"/>
       <c r="V61" s="21">
         <f>SUM(V3:V60)</f>
         <v>33853124</v>
       </c>
     </row>
-    <row r="66" spans="7:21" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="121"/>
+      <c r="B62" s="122"/>
+      <c r="C62" s="122"/>
+      <c r="D62" s="122"/>
+      <c r="E62" s="67"/>
+      <c r="F62" s="21">
+        <f>SUM(F3:F61)</f>
+        <v>105097847.05882354</v>
+      </c>
+      <c r="G62" s="21">
+        <f t="shared" ref="G62:H62" si="23">SUM(G3:G61)</f>
+        <v>19968590.941176467</v>
+      </c>
+      <c r="H62" s="21">
+        <f t="shared" si="23"/>
+        <v>125066438</v>
+      </c>
+    </row>
+    <row r="66" spans="5:21" x14ac:dyDescent="0.3">
+      <c r="E66" s="108"/>
       <c r="U66" s="45"/>
     </row>
-    <row r="68" spans="7:21" x14ac:dyDescent="0.3">
-      <c r="G68" s="11"/>
-    </row>
-    <row r="69" spans="7:21" x14ac:dyDescent="0.3">
-      <c r="G69" s="17"/>
+    <row r="69" spans="5:21" x14ac:dyDescent="0.3">
+      <c r="G69" s="11"/>
+    </row>
+    <row r="70" spans="5:21" x14ac:dyDescent="0.3">
+      <c r="G70" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="J2:Q32" xr:uid="{2822C60C-6EB5-4419-A8A5-7CA3B8AEE8EE}"/>
@@ -4640,15 +4744,15 @@
     <sortCondition ref="S3:S15"/>
   </sortState>
   <mergeCells count="9">
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="J61:M61"/>
+    <mergeCell ref="S1:S2"/>
     <mergeCell ref="T1:V1"/>
     <mergeCell ref="S61:U61"/>
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:Q1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:H1"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="J61:M61"/>
-    <mergeCell ref="S1:S2"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4927,17 +5031,17 @@
     </row>
     <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:14" s="12" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="118" t="s">
+      <c r="A20" s="124" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
-      <c r="G20" s="119"/>
-      <c r="H20" s="119"/>
-      <c r="I20" s="119"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="125"/>
+      <c r="D20" s="125"/>
+      <c r="E20" s="125"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="125"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="125"/>
       <c r="J20" s="13">
         <f>SUM(J2:J19)</f>
         <v>500815</v>
@@ -5234,17 +5338,17 @@
     </row>
     <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:14" s="12" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="118" t="s">
+      <c r="A20" s="124" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
-      <c r="G20" s="119"/>
-      <c r="H20" s="119"/>
-      <c r="I20" s="119"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="125"/>
+      <c r="D20" s="125"/>
+      <c r="E20" s="125"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="125"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="125"/>
       <c r="J20" s="13">
         <f>SUM(J2:J19)</f>
         <v>332408</v>
@@ -5845,17 +5949,17 @@
     </row>
     <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:14" s="12" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="118" t="s">
+      <c r="A20" s="124" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
-      <c r="G20" s="119"/>
-      <c r="H20" s="119"/>
-      <c r="I20" s="119"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="125"/>
+      <c r="D20" s="125"/>
+      <c r="E20" s="125"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="125"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="125"/>
       <c r="J20" s="13">
         <f>SUM(J2:J19)</f>
         <v>1621261</v>
@@ -6400,17 +6504,17 @@
     </row>
     <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:14" s="12" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="118" t="s">
+      <c r="A20" s="124" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
-      <c r="G20" s="119"/>
-      <c r="H20" s="119"/>
-      <c r="I20" s="119"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="125"/>
+      <c r="D20" s="125"/>
+      <c r="E20" s="125"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="125"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="125"/>
       <c r="J20" s="13">
         <f>SUM(J2:J19)</f>
         <v>0</v>
@@ -7059,17 +7163,17 @@
     </row>
     <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:14" s="12" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="118" t="s">
+      <c r="A20" s="124" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
-      <c r="G20" s="119"/>
-      <c r="H20" s="119"/>
-      <c r="I20" s="119"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="125"/>
+      <c r="D20" s="125"/>
+      <c r="E20" s="125"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="125"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="125"/>
       <c r="J20" s="13">
         <f>SUM(J2:J19)</f>
         <v>489210</v>

</xml_diff>